<commit_message>
demo: multi-format samples and regenerate helper after Wave 1
Add deck.pptx, memo.docx, form.pdf; refresh financials with merges/named
ranges; document CLI smoke for new + v0 ops; bake standing demo gate into
the parity plan and AGENTS.md.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo/financials.xlsx
+++ b/demo/financials.xlsx
@@ -10,26 +10,26 @@
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Revenue" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="Rate">Inputs!$B$2</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+  <si>
+    <t>Assumptions</t>
+  </si>
+  <si>
+    <t>Rate</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
   <si>
     <t>Label</t>
-  </si>
-  <si>
-    <t>Value</t>
-  </si>
-  <si>
-    <t>Rate</t>
-  </si>
-  <si>
-    <t>Base</t>
-  </si>
-  <si>
-    <t>Month</t>
   </si>
   <si>
     <t>Amount</t>
@@ -51,8 +51,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -80,8 +88,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -380,16 +389,14 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
+      <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>0.1</v>
@@ -397,13 +404,16 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>100</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -414,16 +424,16 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -431,7 +441,7 @@
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3">
         <v>150</v>
@@ -439,7 +449,7 @@
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <f>B2+B3</f>
@@ -448,7 +458,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5">
         <f>B4*Inputs!B2</f>

</xml_diff>

<commit_message>
feat(xlsx): surface cell number_format and style_id in inspect/read
Parse styles.xml + cell style indices so agents can see percent/currency
formats via inspect style_table and ast_range without a style writer.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo/financials.xlsx
+++ b/demo/financials.xlsx
@@ -51,6 +51,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0%"/>
+    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -88,9 +92,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -398,7 +404,7 @@
       <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="2">
         <v>0.1</v>
       </c>
     </row>
@@ -406,7 +412,7 @@
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>100</v>
       </c>
     </row>
@@ -435,7 +441,7 @@
       <c r="A2" t="s">
         <v>5</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="3">
         <v>100</v>
       </c>
     </row>
@@ -443,7 +449,7 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="3">
         <v>150</v>
       </c>
     </row>
@@ -451,7 +457,7 @@
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="3">
         <f>B2+B3</f>
         <v>0</v>
       </c>
@@ -460,7 +466,7 @@
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="3">
         <f>B4*Inputs!B2</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
feat(xlsx): surgical set_column_width and set_row_height
Agents can adjust worksheet layout via cols/row XML patches without a style engine; other sheets stay byte-identical and merge/set_range paths remain intact.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/demo/financials.xlsx
+++ b/demo/financials.xlsx
@@ -393,8 +393,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" ht="21.75" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -428,6 +432,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="2" width="14.7109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">

</xml_diff>